<commit_message>
Resolve topdown PMU aliases
</commit_message>
<xml_diff>
--- a/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
+++ b/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="L39" s="5">
-        <v>1.78</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="40">
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="L40" s="5">
-        <v>1.86</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="41">
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="L41" s="5">
-        <v>1.94</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="42">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="L42" s="5">
-        <v>2.02</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="43">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="J43" s="5">
-        <v>1.7</v>
+        <v>1.78</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
         </is>
       </c>
       <c r="L43" s="5">
-        <v>2.1</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="44">
@@ -2865,17 +2865,15 @@
         </is>
       </c>
       <c r="J44" s="5">
+        <v>1.46</v>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>L2I_TLB_REFILL_PKI</t>
+        </is>
+      </c>
+      <c r="L44" s="5">
         <v>1.38</v>
-      </c>
-      <c r="K44" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L44" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="45">
@@ -2917,7 +2915,7 @@
         </is>
       </c>
       <c r="J45" s="5">
-        <v>1.46</v>
+        <v>1.54</v>
       </c>
       <c r="K45" s="1" t="inlineStr">
         <is>
@@ -2971,7 +2969,7 @@
         </is>
       </c>
       <c r="J46" s="5">
-        <v>1.54</v>
+        <v>1.62</v>
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
@@ -3029,7 +3027,7 @@
         </is>
       </c>
       <c r="J47" s="5">
-        <v>1.62</v>
+        <v>1.7</v>
       </c>
       <c r="K47" s="1" t="inlineStr">
         <is>
@@ -3323,7 +3321,7 @@
         </is>
       </c>
       <c r="L52" s="5">
-        <v>2.18</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="53">
@@ -3373,7 +3371,7 @@
         </is>
       </c>
       <c r="L53" s="5">
-        <v>2.26</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="54">
@@ -3423,7 +3421,7 @@
         </is>
       </c>
       <c r="L54" s="5">
-        <v>2.34</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="55">
@@ -3473,7 +3471,7 @@
         </is>
       </c>
       <c r="L55" s="5">
-        <v>2.42</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="56">
@@ -3515,7 +3513,7 @@
         </is>
       </c>
       <c r="J56" s="5">
-        <v>2.1</v>
+        <v>2.18</v>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
@@ -3523,7 +3521,7 @@
         </is>
       </c>
       <c r="L56" s="5">
-        <v>2.5</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="57">
@@ -3565,17 +3563,15 @@
         </is>
       </c>
       <c r="J57" s="5">
+        <v>1.86</v>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>L2I_TLB_REFILL_PKI</t>
+        </is>
+      </c>
+      <c r="L57" s="5">
         <v>1.78</v>
-      </c>
-      <c r="K57" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L57" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="58">
@@ -3617,7 +3613,7 @@
         </is>
       </c>
       <c r="J58" s="5">
-        <v>1.86</v>
+        <v>1.94</v>
       </c>
       <c r="K58" s="1" t="inlineStr">
         <is>
@@ -3671,7 +3667,7 @@
         </is>
       </c>
       <c r="J59" s="5">
-        <v>1.94</v>
+        <v>2.02</v>
       </c>
       <c r="K59" s="1" t="inlineStr">
         <is>
@@ -3729,7 +3725,7 @@
         </is>
       </c>
       <c r="J60" s="5">
-        <v>2.02</v>
+        <v>2.1</v>
       </c>
       <c r="K60" s="1" t="inlineStr">
         <is>
@@ -4023,7 +4019,7 @@
         </is>
       </c>
       <c r="L65" s="5">
-        <v>2.58</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="66">
@@ -4073,7 +4069,7 @@
         </is>
       </c>
       <c r="L66" s="5">
-        <v>2.66</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="67">
@@ -4123,7 +4119,7 @@
         </is>
       </c>
       <c r="L67" s="5">
-        <v>2.74</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="68">
@@ -4173,7 +4169,7 @@
         </is>
       </c>
       <c r="L68" s="5">
-        <v>2.82</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="69">
@@ -4215,7 +4211,7 @@
         </is>
       </c>
       <c r="J69" s="5">
-        <v>2.5</v>
+        <v>2.58</v>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
@@ -4223,7 +4219,7 @@
         </is>
       </c>
       <c r="L69" s="5">
-        <v>2.9</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="70">
@@ -4265,17 +4261,15 @@
         </is>
       </c>
       <c r="J70" s="5">
+        <v>2.26</v>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>L2I_TLB_REFILL_PKI</t>
+        </is>
+      </c>
+      <c r="L70" s="5">
         <v>2.18</v>
-      </c>
-      <c r="K70" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L70" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="71">
@@ -4317,7 +4311,7 @@
         </is>
       </c>
       <c r="J71" s="5">
-        <v>2.26</v>
+        <v>2.34</v>
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
@@ -4371,7 +4365,7 @@
         </is>
       </c>
       <c r="J72" s="5">
-        <v>2.34</v>
+        <v>2.42</v>
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
@@ -4429,7 +4423,7 @@
         </is>
       </c>
       <c r="J73" s="5">
-        <v>2.42</v>
+        <v>2.5</v>
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Handle Excel percent formatted Hizee values
</commit_message>
<xml_diff>
--- a/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
+++ b/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,6 +102,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1857,10 +1860,8 @@
           <t>所有进程</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>37.06%</t>
-        </is>
+      <c r="C27" s="7">
+        <v>0.3706</v>
       </c>
       <c r="D27" s="1">
         <v>60.7</v>
@@ -1909,10 +1910,8 @@
           <t>UI进程</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>22.98%</t>
-        </is>
+      <c r="C28" s="7">
+        <v>0.2298</v>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
@@ -1971,10 +1970,8 @@
           <t>render service进程</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>14.08%</t>
-        </is>
+      <c r="C29" s="7">
+        <v>0.1408</v>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
@@ -2033,10 +2030,8 @@
           <t>所有进程</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>44.47%</t>
-        </is>
+      <c r="C30" s="7">
+        <v>0.4447</v>
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
@@ -2093,10 +2088,8 @@
           <t>UI进程</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
-        <is>
-          <t>27.57%</t>
-        </is>
+      <c r="C31" s="7">
+        <v>0.2757</v>
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
@@ -2155,10 +2148,8 @@
           <t>render service进程</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>16.90%</t>
-        </is>
+      <c r="C32" s="7">
+        <v>0.169</v>
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
@@ -2217,10 +2208,8 @@
           <t>所有进程</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
-        <is>
-          <t>54.66%</t>
-        </is>
+      <c r="C33" s="7">
+        <v>0.5466</v>
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
@@ -2277,10 +2266,8 @@
           <t>UI进程</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>33.89%</t>
-        </is>
+      <c r="C34" s="7">
+        <v>0.3389</v>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
@@ -2339,10 +2326,8 @@
           <t>render service进程</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
-        <is>
-          <t>20.77%</t>
-        </is>
+      <c r="C35" s="7">
+        <v>0.2077</v>
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Use target spreadsheet coordinates for imports
</commit_message>
<xml_diff>
--- a/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
+++ b/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
@@ -1815,22 +1815,22 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>DDR平均频率（Mhz）</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>DDR平均频率（Mhz）</t>
+          <t>平均带宽(GB/S)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>平均带宽(GB/S)</t>
+          <t>平均latency(ns)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>平均latency(ns)</t>
+          <t/>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -1869,19 +1869,19 @@
       <c r="E27" s="1">
         <v>985</v>
       </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F27" s="1">
+        <v>2395</v>
       </c>
       <c r="G27" s="1">
-        <v>2395</v>
+        <v>10.4</v>
       </c>
       <c r="H27" s="1">
-        <v>10.4</v>
-      </c>
-      <c r="I27" s="1">
         <v>110.8</v>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
         </is>
       </c>
       <c r="L39" s="5">
-        <v>1.86</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="40">
@@ -2658,7 +2658,7 @@
         </is>
       </c>
       <c r="L40" s="5">
-        <v>1.94</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="41">
@@ -2708,7 +2708,7 @@
         </is>
       </c>
       <c r="L41" s="5">
-        <v>2.02</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="42">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>L2D_TLB_REFILL_PKI</t>
+          <t>L2I_TLB_REFILL_PKI</t>
         </is>
       </c>
       <c r="J42" s="5">
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="L42" s="5">
-        <v>2.1</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="43">
@@ -2800,7 +2800,7 @@
         </is>
       </c>
       <c r="J43" s="5">
-        <v>1.78</v>
+        <v>1.7</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -2808,7 +2808,7 @@
         </is>
       </c>
       <c r="L43" s="5">
-        <v>2.18</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="44">
@@ -2850,15 +2850,17 @@
         </is>
       </c>
       <c r="J44" s="5">
-        <v>1.46</v>
-      </c>
-      <c r="K44" s="5" t="inlineStr">
-        <is>
-          <t>L2I_TLB_REFILL_PKI</t>
-        </is>
-      </c>
-      <c r="L44" s="5">
         <v>1.38</v>
+      </c>
+      <c r="K44" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -2900,7 +2902,7 @@
         </is>
       </c>
       <c r="J45" s="5">
-        <v>1.54</v>
+        <v>1.46</v>
       </c>
       <c r="K45" s="1" t="inlineStr">
         <is>
@@ -2954,7 +2956,7 @@
         </is>
       </c>
       <c r="J46" s="5">
-        <v>1.62</v>
+        <v>1.54</v>
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
@@ -3012,7 +3014,7 @@
         </is>
       </c>
       <c r="J47" s="5">
-        <v>1.7</v>
+        <v>1.62</v>
       </c>
       <c r="K47" s="1" t="inlineStr">
         <is>
@@ -3306,7 +3308,7 @@
         </is>
       </c>
       <c r="L52" s="5">
-        <v>2.26</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="53">
@@ -3356,7 +3358,7 @@
         </is>
       </c>
       <c r="L53" s="5">
-        <v>2.34</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="54">
@@ -3406,7 +3408,7 @@
         </is>
       </c>
       <c r="L54" s="5">
-        <v>2.42</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="55">
@@ -3444,7 +3446,7 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>L2D_TLB_REFILL_PKI</t>
+          <t>L2I_TLB_REFILL_PKI</t>
         </is>
       </c>
       <c r="J55" s="5">
@@ -3456,7 +3458,7 @@
         </is>
       </c>
       <c r="L55" s="5">
-        <v>2.5</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="56">
@@ -3498,7 +3500,7 @@
         </is>
       </c>
       <c r="J56" s="5">
-        <v>2.18</v>
+        <v>2.1</v>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
@@ -3506,7 +3508,7 @@
         </is>
       </c>
       <c r="L56" s="5">
-        <v>2.58</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="57">
@@ -3548,15 +3550,17 @@
         </is>
       </c>
       <c r="J57" s="5">
-        <v>1.86</v>
-      </c>
-      <c r="K57" s="5" t="inlineStr">
-        <is>
-          <t>L2I_TLB_REFILL_PKI</t>
-        </is>
-      </c>
-      <c r="L57" s="5">
         <v>1.78</v>
+      </c>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L57" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -3598,7 +3602,7 @@
         </is>
       </c>
       <c r="J58" s="5">
-        <v>1.94</v>
+        <v>1.86</v>
       </c>
       <c r="K58" s="1" t="inlineStr">
         <is>
@@ -3652,7 +3656,7 @@
         </is>
       </c>
       <c r="J59" s="5">
-        <v>2.02</v>
+        <v>1.94</v>
       </c>
       <c r="K59" s="1" t="inlineStr">
         <is>
@@ -3710,7 +3714,7 @@
         </is>
       </c>
       <c r="J60" s="5">
-        <v>2.1</v>
+        <v>2.02</v>
       </c>
       <c r="K60" s="1" t="inlineStr">
         <is>
@@ -4004,7 +4008,7 @@
         </is>
       </c>
       <c r="L65" s="5">
-        <v>2.66</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="66">
@@ -4054,7 +4058,7 @@
         </is>
       </c>
       <c r="L66" s="5">
-        <v>2.74</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="67">
@@ -4104,7 +4108,7 @@
         </is>
       </c>
       <c r="L67" s="5">
-        <v>2.82</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="68">
@@ -4142,7 +4146,7 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>L2D_TLB_REFILL_PKI</t>
+          <t>L2I_TLB_REFILL_PKI</t>
         </is>
       </c>
       <c r="J68" s="5">
@@ -4154,7 +4158,7 @@
         </is>
       </c>
       <c r="L68" s="5">
-        <v>2.9</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="69">
@@ -4196,7 +4200,7 @@
         </is>
       </c>
       <c r="J69" s="5">
-        <v>2.58</v>
+        <v>2.5</v>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
@@ -4204,7 +4208,7 @@
         </is>
       </c>
       <c r="L69" s="5">
-        <v>2.98</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="70">
@@ -4246,15 +4250,17 @@
         </is>
       </c>
       <c r="J70" s="5">
-        <v>2.26</v>
-      </c>
-      <c r="K70" s="5" t="inlineStr">
-        <is>
-          <t>L2I_TLB_REFILL_PKI</t>
-        </is>
-      </c>
-      <c r="L70" s="5">
         <v>2.18</v>
+      </c>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L70" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -4296,7 +4302,7 @@
         </is>
       </c>
       <c r="J71" s="5">
-        <v>2.34</v>
+        <v>2.26</v>
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
@@ -4350,7 +4356,7 @@
         </is>
       </c>
       <c r="J72" s="5">
-        <v>2.42</v>
+        <v>2.34</v>
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
@@ -4408,7 +4414,7 @@
         </is>
       </c>
       <c r="J73" s="5">
-        <v>2.5</v>
+        <v>2.42</v>
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
@@ -4860,24 +4866,24 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
           <t>LD/ST_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="G81" s="5">
+      <c r="F81" s="5">
         <v>0.72</v>
       </c>
-      <c r="H81" s="5" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>BR_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="I81" s="1">
+      <c r="H81" s="5">
         <v>0.83</v>
+      </c>
+      <c r="I81" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J81" s="1" t="inlineStr">
         <is>
@@ -4914,24 +4920,24 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F82" s="5" t="inlineStr">
-        <is>
           <t>DP_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G82" s="5">
+      <c r="F82" s="5">
         <v>0.94</v>
       </c>
-      <c r="H82" s="5" t="inlineStr">
+      <c r="G82" s="5" t="inlineStr">
         <is>
           <t>VFP_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I82" s="1">
+      <c r="H82" s="5">
         <v>1.05</v>
+      </c>
+      <c r="I82" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J82" s="1" t="inlineStr">
         <is>
@@ -4968,24 +4974,24 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
-        <is>
           <t>ASE_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G83" s="5">
+      <c r="F83" s="5">
         <v>1.16</v>
       </c>
-      <c r="H83" s="5" t="inlineStr">
+      <c r="G83" s="5" t="inlineStr">
         <is>
           <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I83" s="1">
+      <c r="H83" s="5">
         <v>1.27</v>
+      </c>
+      <c r="I83" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
@@ -5022,24 +5028,24 @@
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F84" s="5" t="inlineStr">
-        <is>
           <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G84" s="5">
+      <c r="F84" s="5">
         <v>1.38</v>
       </c>
-      <c r="H84" s="5" t="inlineStr">
+      <c r="G84" s="5" t="inlineStr">
         <is>
           <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I84" s="1">
+      <c r="H84" s="5">
         <v>1.49</v>
+      </c>
+      <c r="I84" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
@@ -5076,24 +5082,24 @@
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F85" s="5" t="inlineStr">
-        <is>
           <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G85" s="5">
+      <c r="F85" s="5">
         <v>1.6</v>
       </c>
-      <c r="H85" s="5" t="inlineStr">
+      <c r="G85" s="5" t="inlineStr">
         <is>
           <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I85" s="1">
+      <c r="H85" s="5">
         <v>1.71</v>
+      </c>
+      <c r="I85" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J85" s="1" t="inlineStr">
         <is>
@@ -5378,24 +5384,24 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
           <t>LD/ST_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="G90" s="5">
+      <c r="F90" s="5">
         <v>0.89</v>
       </c>
-      <c r="H90" s="5" t="inlineStr">
+      <c r="G90" s="5" t="inlineStr">
         <is>
           <t>BR_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="I90" s="1">
+      <c r="H90" s="5">
         <v>1</v>
+      </c>
+      <c r="I90" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J90" s="1" t="inlineStr">
         <is>
@@ -5432,24 +5438,24 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
           <t>DP_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G91" s="5">
+      <c r="F91" s="5">
         <v>1.11</v>
       </c>
-      <c r="H91" s="5" t="inlineStr">
+      <c r="G91" s="5" t="inlineStr">
         <is>
           <t>VFP_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I91" s="1">
+      <c r="H91" s="5">
         <v>1.22</v>
+      </c>
+      <c r="I91" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J91" s="1" t="inlineStr">
         <is>
@@ -5486,24 +5492,24 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
           <t>ASE_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G92" s="5">
+      <c r="F92" s="5">
         <v>1.33</v>
       </c>
-      <c r="H92" s="5" t="inlineStr">
+      <c r="G92" s="5" t="inlineStr">
         <is>
           <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I92" s="1">
+      <c r="H92" s="5">
         <v>1.44</v>
+      </c>
+      <c r="I92" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J92" s="1" t="inlineStr">
         <is>
@@ -5540,24 +5546,24 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
           <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G93" s="5">
+      <c r="F93" s="5">
         <v>1.55</v>
       </c>
-      <c r="H93" s="5" t="inlineStr">
+      <c r="G93" s="5" t="inlineStr">
         <is>
           <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I93" s="1">
+      <c r="H93" s="5">
         <v>1.66</v>
+      </c>
+      <c r="I93" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J93" s="1" t="inlineStr">
         <is>
@@ -5594,24 +5600,24 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
           <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G94" s="5">
+      <c r="F94" s="5">
         <v>1.77</v>
       </c>
-      <c r="H94" s="5" t="inlineStr">
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I94" s="1">
+      <c r="H94" s="5">
         <v>1.88</v>
+      </c>
+      <c r="I94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J94" s="1" t="inlineStr">
         <is>
@@ -5834,24 +5840,24 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
           <t>LD/ST_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="G98" s="5">
+      <c r="F98" s="5">
         <v>1.06</v>
       </c>
-      <c r="H98" s="5" t="inlineStr">
+      <c r="G98" s="5" t="inlineStr">
         <is>
           <t>BR_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="I98" s="1">
+      <c r="H98" s="5">
         <v>1.17</v>
+      </c>
+      <c r="I98" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J98" s="1" t="inlineStr">
         <is>
@@ -5888,24 +5894,24 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F99" s="5" t="inlineStr">
-        <is>
           <t>DP_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G99" s="5">
+      <c r="F99" s="5">
         <v>1.28</v>
       </c>
-      <c r="H99" s="5" t="inlineStr">
+      <c r="G99" s="5" t="inlineStr">
         <is>
           <t>VFP_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I99" s="1">
+      <c r="H99" s="5">
         <v>1.39</v>
+      </c>
+      <c r="I99" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J99" s="1" t="inlineStr">
         <is>
@@ -5942,24 +5948,24 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F100" s="5" t="inlineStr">
-        <is>
           <t>ASE_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G100" s="5">
+      <c r="F100" s="5">
         <v>1.5</v>
       </c>
-      <c r="H100" s="5" t="inlineStr">
+      <c r="G100" s="5" t="inlineStr">
         <is>
           <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I100" s="1">
+      <c r="H100" s="5">
         <v>1.61</v>
+      </c>
+      <c r="I100" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J100" s="1" t="inlineStr">
         <is>
@@ -5996,24 +6002,24 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F101" s="5" t="inlineStr">
-        <is>
           <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G101" s="5">
+      <c r="F101" s="5">
         <v>1.72</v>
       </c>
-      <c r="H101" s="5" t="inlineStr">
+      <c r="G101" s="5" t="inlineStr">
         <is>
           <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I101" s="1">
+      <c r="H101" s="5">
         <v>1.83</v>
+      </c>
+      <c r="I101" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J101" s="1" t="inlineStr">
         <is>
@@ -6050,24 +6056,24 @@
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F102" s="5" t="inlineStr">
-        <is>
           <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
-      <c r="G102" s="5">
+      <c r="F102" s="5">
         <v>1.94</v>
       </c>
-      <c r="H102" s="5" t="inlineStr">
+      <c r="G102" s="5" t="inlineStr">
         <is>
           <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
-      <c r="I102" s="1">
+      <c r="H102" s="5">
         <v>2.05</v>
+      </c>
+      <c r="I102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J102" s="1" t="inlineStr">
         <is>
@@ -6526,12 +6532,12 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libil2cpp.so(37%)</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>Library: libil2cpp.so(37%)</t>
+          <t/>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
@@ -6541,12 +6547,12 @@
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_WaitFence(20.25%)</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_WaitFence(20.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
@@ -6603,12 +6609,12 @@
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_BinderTransact(17.05%)</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_BinderTransact(17.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
@@ -6665,12 +6671,12 @@
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_PhysicsStep(13.85%)</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(13.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
@@ -6712,12 +6718,12 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(30%)</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(30%)</t>
+          <t/>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
@@ -6727,12 +6733,12 @@
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_UpdateScene(20.75%)</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_UpdateScene(20.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
@@ -6789,12 +6795,12 @@
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_TextureUpload(17.55%)</t>
         </is>
       </c>
       <c r="G114" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_TextureUpload(17.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H114" s="1" t="inlineStr">
@@ -6851,12 +6857,12 @@
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_EncodeFrame(14.35%)</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_EncodeFrame(14.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
@@ -6898,12 +6904,12 @@
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(23%)</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(23%)</t>
+          <t/>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
@@ -6913,12 +6919,12 @@
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_BinderTransact(21.25%)</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_BinderTransact(21.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
@@ -6975,12 +6981,12 @@
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_PhysicsStep(18.05%)</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(18.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
@@ -7037,12 +7043,12 @@
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_RenderFrame(14.85%)</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(14.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
@@ -7084,12 +7090,12 @@
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libc.so(38.5%)</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>Library: libc.so(38.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
@@ -7099,12 +7105,12 @@
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_BinderTransact(21.25%)</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_BinderTransact(21.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
@@ -7161,12 +7167,12 @@
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_PhysicsStep(18.05%)</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(18.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
@@ -7223,12 +7229,12 @@
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_RenderFrame(14.85%)</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(14.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
@@ -7270,12 +7276,12 @@
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(31.5%)</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(31.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
@@ -7285,12 +7291,12 @@
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_TextureUpload(21.75%)</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_TextureUpload(21.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
@@ -7347,12 +7353,12 @@
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_EncodeFrame(18.55%)</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_EncodeFrame(18.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
@@ -7409,12 +7415,12 @@
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_ScheduleTask(15.35%)</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_ScheduleTask(15.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
@@ -7456,12 +7462,12 @@
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(24.5%)</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
@@ -7471,12 +7477,12 @@
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_PhysicsStep(22.25%)</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(22.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
@@ -7533,12 +7539,12 @@
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_RenderFrame(19.05%)</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(19.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
@@ -7595,12 +7601,12 @@
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_DoSyscall(15.85%)</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_DoSyscall(15.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
@@ -7642,12 +7648,12 @@
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(40%)</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(40%)</t>
+          <t/>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
@@ -7657,12 +7663,12 @@
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_PhysicsStep(22.25%)</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(22.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
@@ -7719,12 +7725,12 @@
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_RenderFrame(19.05%)</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(19.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
@@ -7781,12 +7787,12 @@
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_DoSyscall(15.85%)</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_DoSyscall(15.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
@@ -7828,12 +7834,12 @@
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(33%)</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(33%)</t>
+          <t/>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
@@ -7843,12 +7849,12 @@
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_EncodeFrame(22.75%)</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_EncodeFrame(22.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
@@ -7905,12 +7911,12 @@
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_ScheduleTask(19.55%)</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_ScheduleTask(19.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
@@ -7967,12 +7973,12 @@
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_WaitFence(16.35%)</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_WaitFence(16.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
@@ -8014,12 +8020,12 @@
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(26%)</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(26%)</t>
+          <t/>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
@@ -8029,12 +8035,12 @@
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_RenderFrame(23.25%)</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(23.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
@@ -8091,12 +8097,12 @@
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_DoSyscall(20.05%)</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_DoSyscall(20.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
@@ -8153,12 +8159,12 @@
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: cycle_UpdateScene(16.85%)</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_UpdateScene(16.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
@@ -8262,12 +8268,12 @@
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libc.so(37%)</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>Library: libc.so(37%)</t>
+          <t/>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
@@ -8277,12 +8283,12 @@
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_UpdateScene(20.25%)</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_UpdateScene(20.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
@@ -8339,12 +8345,12 @@
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_TextureUpload(17.05%)</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_TextureUpload(17.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
@@ -8401,12 +8407,12 @@
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_EncodeFrame(13.85%)</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(13.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H140" s="1" t="inlineStr">
@@ -8448,12 +8454,12 @@
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(30%)</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(30%)</t>
+          <t/>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
@@ -8463,12 +8469,12 @@
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_BinderTransact(20.75%)</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_BinderTransact(20.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H141" s="1" t="inlineStr">
@@ -8525,12 +8531,12 @@
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_PhysicsStep(17.55%)</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_PhysicsStep(17.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H142" s="1" t="inlineStr">
@@ -8587,12 +8593,12 @@
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_RenderFrame(14.35%)</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_RenderFrame(14.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H143" s="1" t="inlineStr">
@@ -8634,12 +8640,12 @@
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(23%)</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(23%)</t>
+          <t/>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
@@ -8649,12 +8655,12 @@
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_TextureUpload(21.25%)</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_TextureUpload(21.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H144" s="1" t="inlineStr">
@@ -8711,12 +8717,12 @@
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_EncodeFrame(18.05%)</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(18.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H145" s="1" t="inlineStr">
@@ -8773,12 +8779,12 @@
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_ScheduleTask(14.85%)</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(14.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H146" s="1" t="inlineStr">
@@ -8820,12 +8826,12 @@
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(38.5%)</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(38.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
@@ -8835,12 +8841,12 @@
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_TextureUpload(21.25%)</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_TextureUpload(21.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr">
@@ -8897,12 +8903,12 @@
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_EncodeFrame(18.05%)</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(18.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H148" s="1" t="inlineStr">
@@ -8959,12 +8965,12 @@
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_ScheduleTask(14.85%)</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(14.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H149" s="1" t="inlineStr">
@@ -9006,12 +9012,12 @@
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(31.5%)</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(31.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
@@ -9021,12 +9027,12 @@
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_PhysicsStep(21.75%)</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_PhysicsStep(21.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H150" s="1" t="inlineStr">
@@ -9083,12 +9089,12 @@
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_RenderFrame(18.55%)</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_RenderFrame(18.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H151" s="1" t="inlineStr">
@@ -9145,12 +9151,12 @@
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_DoSyscall(15.35%)</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_DoSyscall(15.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H152" s="1" t="inlineStr">
@@ -9192,12 +9198,12 @@
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(24.5%)</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
@@ -9207,12 +9213,12 @@
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_EncodeFrame(22.25%)</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(22.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H153" s="1" t="inlineStr">
@@ -9269,12 +9275,12 @@
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_ScheduleTask(19.05%)</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(19.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H154" s="1" t="inlineStr">
@@ -9331,12 +9337,12 @@
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_WaitFence(15.85%)</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_WaitFence(15.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H155" s="1" t="inlineStr">
@@ -9378,12 +9384,12 @@
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(40%)</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(40%)</t>
+          <t/>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
@@ -9393,12 +9399,12 @@
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_EncodeFrame(22.25%)</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(22.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H156" s="1" t="inlineStr">
@@ -9455,12 +9461,12 @@
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_ScheduleTask(19.05%)</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(19.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H157" s="1" t="inlineStr">
@@ -9517,12 +9523,12 @@
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_WaitFence(15.85%)</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_WaitFence(15.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H158" s="1" t="inlineStr">
@@ -9564,12 +9570,12 @@
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(33%)</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(33%)</t>
+          <t/>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
@@ -9579,12 +9585,12 @@
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_RenderFrame(22.75%)</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_RenderFrame(22.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H159" s="1" t="inlineStr">
@@ -9641,12 +9647,12 @@
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_DoSyscall(19.55%)</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_DoSyscall(19.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H160" s="1" t="inlineStr">
@@ -9703,12 +9709,12 @@
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_UpdateScene(16.35%)</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_UpdateScene(16.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H161" s="1" t="inlineStr">
@@ -9750,12 +9756,12 @@
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libhwui.so(26%)</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>Library: libhwui.so(26%)</t>
+          <t/>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
@@ -9765,12 +9771,12 @@
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_ScheduleTask(23.25%)</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(23.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H162" s="1" t="inlineStr">
@@ -9827,12 +9833,12 @@
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_WaitFence(20.05%)</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_WaitFence(20.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H163" s="1" t="inlineStr">
@@ -9889,12 +9895,12 @@
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: fe_BinderTransact(16.85%)</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_BinderTransact(16.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H164" s="1" t="inlineStr">
@@ -9998,12 +10004,12 @@
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(37%)</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(37%)</t>
+          <t/>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
@@ -10013,12 +10019,12 @@
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_BinderTransact(20.25%)</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>Function: be_BinderTransact(20.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H166" s="1" t="inlineStr">
@@ -10075,12 +10081,12 @@
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_PhysicsStep(17.05%)</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>Function: be_PhysicsStep(17.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H167" s="1" t="inlineStr">
@@ -10137,12 +10143,12 @@
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_RenderFrame(13.85%)</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(13.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H168" s="1" t="inlineStr">
@@ -10184,12 +10190,12 @@
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(30%)</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(30%)</t>
+          <t/>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
@@ -10199,12 +10205,12 @@
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_TextureUpload(20.75%)</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>Function: be_TextureUpload(20.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H169" s="1" t="inlineStr">
@@ -10261,12 +10267,12 @@
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_EncodeFrame(17.55%)</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>Function: be_EncodeFrame(17.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H170" s="1" t="inlineStr">
@@ -10323,12 +10329,12 @@
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_ScheduleTask(14.35%)</t>
         </is>
       </c>
       <c r="G171" s="1" t="inlineStr">
         <is>
-          <t>Function: be_ScheduleTask(14.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H171" s="1" t="inlineStr">
@@ -10370,12 +10376,12 @@
       </c>
       <c r="C172" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(23%)</t>
         </is>
       </c>
       <c r="D172" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(23%)</t>
+          <t/>
         </is>
       </c>
       <c r="E172" s="1" t="inlineStr">
@@ -10385,12 +10391,12 @@
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_PhysicsStep(21.25%)</t>
         </is>
       </c>
       <c r="G172" s="1" t="inlineStr">
         <is>
-          <t>Function: be_PhysicsStep(21.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H172" s="1" t="inlineStr">
@@ -10447,12 +10453,12 @@
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_RenderFrame(18.05%)</t>
         </is>
       </c>
       <c r="G173" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(18.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H173" s="1" t="inlineStr">
@@ -10509,12 +10515,12 @@
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_DoSyscall(14.85%)</t>
         </is>
       </c>
       <c r="G174" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(14.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H174" s="1" t="inlineStr">
@@ -10556,12 +10562,12 @@
       </c>
       <c r="C175" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(38.5%)</t>
         </is>
       </c>
       <c r="D175" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(38.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E175" s="1" t="inlineStr">
@@ -10571,12 +10577,12 @@
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_PhysicsStep(21.25%)</t>
         </is>
       </c>
       <c r="G175" s="1" t="inlineStr">
         <is>
-          <t>Function: be_PhysicsStep(21.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H175" s="1" t="inlineStr">
@@ -10633,12 +10639,12 @@
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_RenderFrame(18.05%)</t>
         </is>
       </c>
       <c r="G176" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(18.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H176" s="1" t="inlineStr">
@@ -10695,12 +10701,12 @@
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_DoSyscall(14.85%)</t>
         </is>
       </c>
       <c r="G177" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(14.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H177" s="1" t="inlineStr">
@@ -10742,12 +10748,12 @@
       </c>
       <c r="C178" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(31.5%)</t>
         </is>
       </c>
       <c r="D178" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(31.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E178" s="1" t="inlineStr">
@@ -10757,12 +10763,12 @@
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_EncodeFrame(21.75%)</t>
         </is>
       </c>
       <c r="G178" s="1" t="inlineStr">
         <is>
-          <t>Function: be_EncodeFrame(21.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H178" s="1" t="inlineStr">
@@ -10819,12 +10825,12 @@
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_ScheduleTask(18.55%)</t>
         </is>
       </c>
       <c r="G179" s="1" t="inlineStr">
         <is>
-          <t>Function: be_ScheduleTask(18.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H179" s="1" t="inlineStr">
@@ -10881,12 +10887,12 @@
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_WaitFence(15.35%)</t>
         </is>
       </c>
       <c r="G180" s="1" t="inlineStr">
         <is>
-          <t>Function: be_WaitFence(15.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H180" s="1" t="inlineStr">
@@ -10928,12 +10934,12 @@
       </c>
       <c r="C181" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libhwui.so(24.5%)</t>
         </is>
       </c>
       <c r="D181" s="1" t="inlineStr">
         <is>
-          <t>Library: libhwui.so(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="E181" s="1" t="inlineStr">
@@ -10943,12 +10949,12 @@
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_RenderFrame(22.25%)</t>
         </is>
       </c>
       <c r="G181" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(22.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H181" s="1" t="inlineStr">
@@ -11005,12 +11011,12 @@
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_DoSyscall(19.05%)</t>
         </is>
       </c>
       <c r="G182" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(19.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H182" s="1" t="inlineStr">
@@ -11067,12 +11073,12 @@
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_UpdateScene(15.85%)</t>
         </is>
       </c>
       <c r="G183" s="1" t="inlineStr">
         <is>
-          <t>Function: be_UpdateScene(15.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H183" s="1" t="inlineStr">
@@ -11114,12 +11120,12 @@
       </c>
       <c r="C184" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(40%)</t>
         </is>
       </c>
       <c r="D184" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(40%)</t>
+          <t/>
         </is>
       </c>
       <c r="E184" s="1" t="inlineStr">
@@ -11129,12 +11135,12 @@
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_RenderFrame(22.25%)</t>
         </is>
       </c>
       <c r="G184" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(22.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H184" s="1" t="inlineStr">
@@ -11191,12 +11197,12 @@
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_DoSyscall(19.05%)</t>
         </is>
       </c>
       <c r="G185" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(19.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H185" s="1" t="inlineStr">
@@ -11253,12 +11259,12 @@
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_UpdateScene(15.85%)</t>
         </is>
       </c>
       <c r="G186" s="1" t="inlineStr">
         <is>
-          <t>Function: be_UpdateScene(15.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H186" s="1" t="inlineStr">
@@ -11300,12 +11306,12 @@
       </c>
       <c r="C187" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(33%)</t>
         </is>
       </c>
       <c r="D187" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(33%)</t>
+          <t/>
         </is>
       </c>
       <c r="E187" s="1" t="inlineStr">
@@ -11315,12 +11321,12 @@
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_ScheduleTask(22.75%)</t>
         </is>
       </c>
       <c r="G187" s="1" t="inlineStr">
         <is>
-          <t>Function: be_ScheduleTask(22.75%)</t>
+          <t/>
         </is>
       </c>
       <c r="H187" s="1" t="inlineStr">
@@ -11377,12 +11383,12 @@
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_WaitFence(19.55%)</t>
         </is>
       </c>
       <c r="G188" s="1" t="inlineStr">
         <is>
-          <t>Function: be_WaitFence(19.55%)</t>
+          <t/>
         </is>
       </c>
       <c r="H188" s="1" t="inlineStr">
@@ -11439,12 +11445,12 @@
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_BinderTransact(16.35%)</t>
         </is>
       </c>
       <c r="G189" s="1" t="inlineStr">
         <is>
-          <t>Function: be_BinderTransact(16.35%)</t>
+          <t/>
         </is>
       </c>
       <c r="H189" s="1" t="inlineStr">
@@ -11486,12 +11492,12 @@
       </c>
       <c r="C190" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libart.so(26%)</t>
         </is>
       </c>
       <c r="D190" s="1" t="inlineStr">
         <is>
-          <t>Library: libart.so(26%)</t>
+          <t/>
         </is>
       </c>
       <c r="E190" s="1" t="inlineStr">
@@ -11501,12 +11507,12 @@
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_DoSyscall(23.25%)</t>
         </is>
       </c>
       <c r="G190" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(23.25%)</t>
+          <t/>
         </is>
       </c>
       <c r="H190" s="1" t="inlineStr">
@@ -11563,12 +11569,12 @@
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_UpdateScene(20.05%)</t>
         </is>
       </c>
       <c r="G191" s="1" t="inlineStr">
         <is>
-          <t>Function: be_UpdateScene(20.05%)</t>
+          <t/>
         </is>
       </c>
       <c r="H191" s="1" t="inlineStr">
@@ -11625,12 +11631,12 @@
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Function: be_TextureUpload(16.85%)</t>
         </is>
       </c>
       <c r="G192" s="1" t="inlineStr">
         <is>
-          <t>Function: be_TextureUpload(16.85%)</t>
+          <t/>
         </is>
       </c>
       <c r="H192" s="1" t="inlineStr">
@@ -11660,7 +11666,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="95">
+  <mergeCells count="94">
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:D3"/>
@@ -11675,25 +11681,24 @@
     <mergeCell ref="D8:F25"/>
     <mergeCell ref="G8:I25"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="E26:F26"/>
     <mergeCell ref="A27:A29"/>
     <mergeCell ref="D27:D29"/>
-    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="F27:F29"/>
     <mergeCell ref="G27:G29"/>
     <mergeCell ref="H27:H29"/>
-    <mergeCell ref="I27:I29"/>
     <mergeCell ref="A30:A32"/>
     <mergeCell ref="D30:D32"/>
-    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="F30:F32"/>
     <mergeCell ref="G30:G32"/>
     <mergeCell ref="H30:H32"/>
-    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A33:A35"/>
     <mergeCell ref="D33:D35"/>
-    <mergeCell ref="E33:F35"/>
+    <mergeCell ref="E33:E35"/>
+    <mergeCell ref="F33:F35"/>
     <mergeCell ref="G33:G35"/>
     <mergeCell ref="H33:H35"/>
-    <mergeCell ref="I33:I35"/>
     <mergeCell ref="A37:L37"/>
     <mergeCell ref="A38:L38"/>
     <mergeCell ref="A48:L48"/>
@@ -11718,44 +11723,44 @@
     <mergeCell ref="A107:B107"/>
     <mergeCell ref="A108:L108"/>
     <mergeCell ref="A109:L109"/>
-    <mergeCell ref="D110:F112"/>
-    <mergeCell ref="D113:F115"/>
-    <mergeCell ref="D116:F118"/>
-    <mergeCell ref="A110:C118"/>
-    <mergeCell ref="D119:F121"/>
-    <mergeCell ref="D122:F124"/>
-    <mergeCell ref="D125:F127"/>
-    <mergeCell ref="A119:C127"/>
-    <mergeCell ref="D128:F130"/>
-    <mergeCell ref="D131:F133"/>
-    <mergeCell ref="D134:F136"/>
-    <mergeCell ref="A128:C136"/>
+    <mergeCell ref="C110:E112"/>
+    <mergeCell ref="C113:E115"/>
+    <mergeCell ref="C116:E118"/>
+    <mergeCell ref="A110:B118"/>
+    <mergeCell ref="C119:E121"/>
+    <mergeCell ref="C122:E124"/>
+    <mergeCell ref="C125:E127"/>
+    <mergeCell ref="A119:B127"/>
+    <mergeCell ref="C128:E130"/>
+    <mergeCell ref="C131:E133"/>
+    <mergeCell ref="C134:E136"/>
+    <mergeCell ref="A128:B136"/>
     <mergeCell ref="A137:L137"/>
-    <mergeCell ref="D138:F140"/>
-    <mergeCell ref="D141:F143"/>
-    <mergeCell ref="D144:F146"/>
-    <mergeCell ref="A138:C146"/>
-    <mergeCell ref="D147:F149"/>
-    <mergeCell ref="D150:F152"/>
-    <mergeCell ref="D153:F155"/>
-    <mergeCell ref="A147:C155"/>
-    <mergeCell ref="D156:F158"/>
-    <mergeCell ref="D159:F161"/>
-    <mergeCell ref="D162:F164"/>
-    <mergeCell ref="A156:C164"/>
+    <mergeCell ref="C138:E140"/>
+    <mergeCell ref="C141:E143"/>
+    <mergeCell ref="C144:E146"/>
+    <mergeCell ref="A138:B146"/>
+    <mergeCell ref="C147:E149"/>
+    <mergeCell ref="C150:E152"/>
+    <mergeCell ref="C153:E155"/>
+    <mergeCell ref="A147:B155"/>
+    <mergeCell ref="C156:E158"/>
+    <mergeCell ref="C159:E161"/>
+    <mergeCell ref="C162:E164"/>
+    <mergeCell ref="A156:B164"/>
     <mergeCell ref="A165:L165"/>
-    <mergeCell ref="D166:F168"/>
-    <mergeCell ref="D169:F171"/>
-    <mergeCell ref="D172:F174"/>
-    <mergeCell ref="A166:C174"/>
-    <mergeCell ref="D175:F177"/>
-    <mergeCell ref="D178:F180"/>
-    <mergeCell ref="D181:F183"/>
-    <mergeCell ref="A175:C183"/>
-    <mergeCell ref="D184:F186"/>
-    <mergeCell ref="D187:F189"/>
-    <mergeCell ref="D190:F192"/>
-    <mergeCell ref="A184:C192"/>
+    <mergeCell ref="C166:E168"/>
+    <mergeCell ref="C169:E171"/>
+    <mergeCell ref="C172:E174"/>
+    <mergeCell ref="A166:B174"/>
+    <mergeCell ref="C175:E177"/>
+    <mergeCell ref="C178:E180"/>
+    <mergeCell ref="C181:E183"/>
+    <mergeCell ref="A175:B183"/>
+    <mergeCell ref="C184:E186"/>
+    <mergeCell ref="C187:E189"/>
+    <mergeCell ref="C190:E192"/>
+    <mergeCell ref="A184:B192"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Use fixed target coordinates for source import
</commit_message>
<xml_diff>
--- a/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
+++ b/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
       <c r="D81" s="5">
-        <v>2.43</v>
+        <v>4.29</v>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
@@ -4874,11 +4874,11 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
       <c r="H81" s="5">
-        <v>0.83</v>
+        <v>1.49</v>
       </c>
       <c r="I81" s="1" t="inlineStr">
         <is>
@@ -4904,35 +4904,35 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="B82" s="5">
-        <v>2.74</v>
+        <v>2.43</v>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
+          <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
       <c r="D82" s="5">
-        <v>3.05</v>
+        <v>3.98</v>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="F82" s="5">
-        <v>0.94</v>
+        <v>0.83</v>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
+          <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
       <c r="H82" s="5">
-        <v>1.05</v>
+        <v>1.38</v>
       </c>
       <c r="I82" s="1" t="inlineStr">
         <is>
@@ -4958,35 +4958,35 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>ASE_SPEC_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B83" s="5">
-        <v>3.36</v>
+        <v>2.74</v>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>SVE_INST_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="D83" s="5">
-        <v>3.67</v>
+        <v>4.91</v>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>ASE_SPEC_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F83" s="5">
-        <v>1.16</v>
+        <v>0.94</v>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>SVE_INST_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="H83" s="5">
-        <v>1.27</v>
+        <v>1.71</v>
       </c>
       <c r="I83" s="1" t="inlineStr">
         <is>
@@ -5012,35 +5012,35 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>ASE_SPEC_PKI</t>
         </is>
       </c>
       <c r="B84" s="5">
-        <v>3.98</v>
+        <v>3.36</v>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>ATOMIC/CAS_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="D84" s="5">
-        <v>4.29</v>
+        <v>4.6</v>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>ASE_SPEC_PKI</t>
         </is>
       </c>
       <c r="F84" s="5">
-        <v>1.38</v>
+        <v>1.16</v>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>ATOMIC/CAS_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="H84" s="5">
-        <v>1.49</v>
+        <v>1.6</v>
       </c>
       <c r="I84" s="1" t="inlineStr">
         <is>
@@ -5066,35 +5066,35 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
+          <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
       <c r="B85" s="5">
-        <v>4.6</v>
+        <v>3.67</v>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="D85" s="5">
-        <v>4.91</v>
+        <v>3.05</v>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
+          <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
       <c r="F85" s="5">
-        <v>1.6</v>
+        <v>1.27</v>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="H85" s="5">
-        <v>1.71</v>
+        <v>1.05</v>
       </c>
       <c r="I85" s="1" t="inlineStr">
         <is>
@@ -5180,169 +5180,161 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K87" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L87" s="1" t="inlineStr">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>RenderThread线程</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>RenderThread线程</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L88" s="2" t="inlineStr">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I88" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J88" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K88" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L88" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>Kernel</t>
-        </is>
-      </c>
-      <c r="F89" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G89" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H89" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="B89" s="5">
+        <v>2.6</v>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>ATOMIC/CAS_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D89" s="5">
+        <v>4.77</v>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="F89" s="5">
+        <v>0.89</v>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>ATOMIC/CAS_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="H89" s="5">
+        <v>1.66</v>
       </c>
       <c r="I89" s="1" t="inlineStr">
         <is>
@@ -5368,35 +5360,35 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="B90" s="5">
-        <v>2.6</v>
+        <v>2.91</v>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D90" s="5">
+        <v>4.46</v>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
           <t>BR_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="D90" s="5">
-        <v>2.91</v>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>LD/ST_RETIRED_PKI</t>
-        </is>
-      </c>
       <c r="F90" s="5">
-        <v>0.89</v>
+        <v>1</v>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
       <c r="H90" s="5">
-        <v>1</v>
+        <v>1.55</v>
       </c>
       <c r="I90" s="1" t="inlineStr">
         <is>
@@ -5430,11 +5422,11 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="D91" s="5">
-        <v>3.53</v>
+        <v>5.39</v>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
@@ -5446,11 +5438,11 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="H91" s="5">
-        <v>1.22</v>
+        <v>1.88</v>
       </c>
       <c r="I91" s="1" t="inlineStr">
         <is>
@@ -5484,11 +5476,11 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>SVE_INST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="D92" s="5">
-        <v>4.15</v>
+        <v>5.08</v>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
@@ -5500,11 +5492,11 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>SVE_INST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="H92" s="5">
-        <v>1.44</v>
+        <v>1.77</v>
       </c>
       <c r="I92" s="1" t="inlineStr">
         <is>
@@ -5530,275 +5522,275 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
       <c r="B93" s="5">
-        <v>4.46</v>
+        <v>4.15</v>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
+          <t>VFP_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D93" s="5">
+        <v>3.53</v>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>SVE_INST_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="F93" s="5">
+        <v>1.44</v>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>VFP_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="H93" s="5">
+        <v>1.22</v>
+      </c>
+      <c r="I93" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J93" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K93" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L93" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L94" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>BinderWorker线程</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I96" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J96" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K96" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L96" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="B97" s="5">
+        <v>3.08</v>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
           <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
-      <c r="D93" s="5">
-        <v>4.77</v>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>LD/STREX_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="F93" s="5">
-        <v>1.55</v>
-      </c>
-      <c r="G93" s="5" t="inlineStr">
+      <c r="D97" s="5">
+        <v>5.25</v>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="F97" s="5">
+        <v>1.06</v>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>ATOMIC/CAS_SPEC_PKI</t>
         </is>
       </c>
-      <c r="H93" s="5">
-        <v>1.66</v>
-      </c>
-      <c r="I93" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J93" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K93" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L93" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
-        <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="B94" s="5">
-        <v>5.08</v>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D94" s="5">
-        <v>5.39</v>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="F94" s="5">
-        <v>1.77</v>
-      </c>
-      <c r="G94" s="5" t="inlineStr">
-        <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H94" s="5">
-        <v>1.88</v>
-      </c>
-      <c r="I94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L95" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>BinderWorker线程</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L96" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr">
-        <is>
-          <t>Kernel</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G97" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H97" s="5">
+        <v>1.83</v>
       </c>
       <c r="I97" s="1" t="inlineStr">
         <is>
@@ -5824,35 +5816,35 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="B98" s="5">
-        <v>3.08</v>
+        <v>3.39</v>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D98" s="5">
+        <v>4.94</v>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
           <t>BR_RETIRED_PKI</t>
         </is>
       </c>
-      <c r="D98" s="5">
-        <v>3.39</v>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>LD/ST_RETIRED_PKI</t>
-        </is>
-      </c>
       <c r="F98" s="5">
-        <v>1.06</v>
+        <v>1.17</v>
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>LD/STREX_SPEC_PKI</t>
         </is>
       </c>
       <c r="H98" s="5">
-        <v>1.17</v>
+        <v>1.72</v>
       </c>
       <c r="I98" s="1" t="inlineStr">
         <is>
@@ -5886,11 +5878,11 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="D99" s="5">
-        <v>4.01</v>
+        <v>5.87</v>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
@@ -5902,11 +5894,11 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="H99" s="5">
-        <v>1.39</v>
+        <v>2.05</v>
       </c>
       <c r="I99" s="1" t="inlineStr">
         <is>
@@ -5940,11 +5932,11 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>SVE_INST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="D100" s="5">
-        <v>4.63</v>
+        <v>5.56</v>
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
@@ -5956,11 +5948,11 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>SVE_INST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="H100" s="5">
-        <v>1.61</v>
+        <v>1.94</v>
       </c>
       <c r="I100" s="1" t="inlineStr">
         <is>
@@ -5986,35 +5978,35 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
       <c r="B101" s="5">
-        <v>4.94</v>
+        <v>4.63</v>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>ATOMIC/CAS_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="D101" s="5">
-        <v>5.25</v>
+        <v>4.01</v>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>SVE_INST_SPEC_PKI</t>
         </is>
       </c>
       <c r="F101" s="5">
-        <v>1.72</v>
+        <v>1.61</v>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>ATOMIC/CAS_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="H101" s="5">
-        <v>1.83</v>
+        <v>1.39</v>
       </c>
       <c r="I101" s="1" t="inlineStr">
         <is>
@@ -6038,37 +6030,45 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="B102" s="5">
-        <v>5.56</v>
-      </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D102" s="5">
-        <v>5.87</v>
-      </c>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="F102" s="5">
-        <v>1.94</v>
-      </c>
-      <c r="G102" s="5" t="inlineStr">
-        <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H102" s="5">
-        <v>2.05</v>
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H102" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I102" s="1" t="inlineStr">
         <is>
@@ -6154,44 +6154,42 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="inlineStr">
-        <is>
-          <t>线程名</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C104" s="3" t="inlineStr">
-        <is>
-          <t>系统调用密度（每千万条指令）</t>
-        </is>
-      </c>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>TOP1系统调用及占比</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="inlineStr">
-        <is>
-          <t>TOP2系统调用及占比</t>
-        </is>
-      </c>
-      <c r="F104" s="3" t="inlineStr">
-        <is>
-          <t>TOP3系统调用及占比</t>
-        </is>
-      </c>
-      <c r="G104" s="3" t="inlineStr">
-        <is>
-          <t>TOP4系统调用及占比</t>
-        </is>
-      </c>
-      <c r="H104" s="3" t="inlineStr">
-        <is>
-          <t>TOP5系统调用及占比</t>
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>UnityMain线程</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C104" s="1">
+        <v>66</v>
+      </c>
+      <c r="D104" s="1" t="inlineStr">
+        <is>
+          <t>43_nanosleep(26.67%)</t>
+        </is>
+      </c>
+      <c r="E104" s="1" t="inlineStr">
+        <is>
+          <t>62_close(19.56%)</t>
+        </is>
+      </c>
+      <c r="F104" s="1" t="inlineStr">
+        <is>
+          <t>81_write(16.47%)</t>
+        </is>
+      </c>
+      <c r="G104" s="1" t="inlineStr">
+        <is>
+          <t>100_recvmsg(16.02%)</t>
+        </is>
+      </c>
+      <c r="H104" s="1" t="inlineStr">
+        <is>
+          <t>119_clock_gettime(5.9%)</t>
         </is>
       </c>
       <c r="I104" s="1" t="inlineStr">
@@ -6218,7 +6216,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>UnityMain线程</t>
+          <t>RenderThread线程</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -6227,31 +6225,31 @@
         </is>
       </c>
       <c r="C105" s="1">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>43_nanosleep(26.67%)</t>
+          <t>44_sendmsg(26.55%)</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>62_close(19.56%)</t>
+          <t>63_ioctl(21.72%)</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>81_write(16.47%)</t>
+          <t>82_openat(16.89%)</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>100_recvmsg(16.02%)</t>
+          <t>101_prctl(8.39%)</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>119_clock_gettime(5.9%)</t>
+          <t>120_mmap(7.84%)</t>
         </is>
       </c>
       <c r="I105" s="1" t="inlineStr">
@@ -6278,7 +6276,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>RenderThread线程</t>
+          <t>BinderWorker线程</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -6287,31 +6285,31 @@
         </is>
       </c>
       <c r="C106" s="1">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>44_sendmsg(26.55%)</t>
+          <t>45_poll(25.45%)</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>63_ioctl(21.72%)</t>
+          <t>64_mprotect(20.8%)</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>82_openat(16.89%)</t>
+          <t>83_futex(20.18%)</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>101_prctl(8.39%)</t>
+          <t>102_close(14.3%)</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>120_mmap(7.84%)</t>
+          <t>121_getpid(3.62%)</t>
         </is>
       </c>
       <c r="I106" s="1" t="inlineStr">
@@ -6338,7 +6336,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>BinderWorker线程</t>
+          <t/>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -6346,32 +6344,34 @@
           <t/>
         </is>
       </c>
-      <c r="C107" s="1">
-        <v>92</v>
+      <c r="C107" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>45_poll(25.45%)</t>
+          <t/>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>64_mprotect(20.8%)</t>
+          <t/>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>83_futex(20.18%)</t>
+          <t/>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>102_close(14.3%)</t>
+          <t/>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>121_getpid(3.62%)</t>
+          <t/>
         </is>
       </c>
       <c r="I107" s="1" t="inlineStr">
@@ -6398,7 +6398,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>6. 热点SO及函数&amp;Bound SO及函数</t>
+          <t>CYCLE</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -6458,62 +6458,62 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>CYCLE</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K109" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L109" s="2" t="inlineStr">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>UnityMain(38.7%)</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>Library: libil2cpp.so(37%)</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F109" s="1" t="inlineStr">
+        <is>
+          <t>Function: cycle_WaitFence(20.25%)</t>
+        </is>
+      </c>
+      <c r="G109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K109" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L109" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -6522,7 +6522,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>UnityMain(38.7%)</t>
+          <t/>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>Library: libil2cpp.so(37%)</t>
+          <t/>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_WaitFence(20.25%)</t>
+          <t>Function: cycle_BinderTransact(17.05%)</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_BinderTransact(17.05%)</t>
+          <t>Function: cycle_PhysicsStep(13.85%)</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(30%)</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
@@ -6671,7 +6671,7 @@
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(13.85%)</t>
+          <t>Function: cycle_UpdateScene(20.75%)</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(30%)</t>
+          <t/>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_UpdateScene(20.75%)</t>
+          <t>Function: cycle_TextureUpload(17.55%)</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
@@ -6795,7 +6795,7 @@
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_TextureUpload(17.55%)</t>
+          <t>Function: cycle_EncodeFrame(14.35%)</t>
         </is>
       </c>
       <c r="G114" s="1" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(23%)</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_EncodeFrame(14.35%)</t>
+          <t>Function: cycle_BinderTransact(21.25%)</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
@@ -6904,7 +6904,7 @@
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(23%)</t>
+          <t/>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
@@ -6919,7 +6919,7 @@
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_BinderTransact(21.25%)</t>
+          <t>Function: cycle_PhysicsStep(18.05%)</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(18.05%)</t>
+          <t>Function: cycle_RenderFrame(14.85%)</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
@@ -7018,7 +7018,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>RenderThread(31.6%)</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libc.so(38.5%)</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(14.85%)</t>
+          <t>Function: cycle_BinderTransact(21.25%)</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
@@ -7080,7 +7080,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>RenderThread(31.6%)</t>
+          <t/>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -7090,7 +7090,7 @@
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>Library: libc.so(38.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_BinderTransact(21.25%)</t>
+          <t>Function: cycle_PhysicsStep(18.05%)</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(18.05%)</t>
+          <t>Function: cycle_RenderFrame(14.85%)</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(31.5%)</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
@@ -7229,7 +7229,7 @@
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(14.85%)</t>
+          <t>Function: cycle_TextureUpload(21.75%)</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(31.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_TextureUpload(21.75%)</t>
+          <t>Function: cycle_EncodeFrame(18.55%)</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_EncodeFrame(18.55%)</t>
+          <t>Function: cycle_ScheduleTask(15.35%)</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
@@ -7400,7 +7400,7 @@
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(24.5%)</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
@@ -7415,7 +7415,7 @@
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_ScheduleTask(15.35%)</t>
+          <t>Function: cycle_PhysicsStep(22.25%)</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
@@ -7462,7 +7462,7 @@
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
@@ -7477,7 +7477,7 @@
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(22.25%)</t>
+          <t>Function: cycle_RenderFrame(19.05%)</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(19.05%)</t>
+          <t>Function: cycle_DoSyscall(15.85%)</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
@@ -7576,7 +7576,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>BinderWorker(24.5%)</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(40%)</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_DoSyscall(15.85%)</t>
+          <t>Function: cycle_PhysicsStep(22.25%)</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
@@ -7638,7 +7638,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>BinderWorker(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(40%)</t>
+          <t/>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_PhysicsStep(22.25%)</t>
+          <t>Function: cycle_RenderFrame(19.05%)</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(19.05%)</t>
+          <t>Function: cycle_DoSyscall(15.85%)</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(33%)</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_DoSyscall(15.85%)</t>
+          <t>Function: cycle_EncodeFrame(22.75%)</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(33%)</t>
+          <t/>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_EncodeFrame(22.75%)</t>
+          <t>Function: cycle_ScheduleTask(19.55%)</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_ScheduleTask(19.55%)</t>
+          <t>Function: cycle_WaitFence(16.35%)</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(26%)</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_WaitFence(16.35%)</t>
+          <t>Function: cycle_RenderFrame(23.25%)</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(26%)</t>
+          <t/>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
@@ -8035,7 +8035,7 @@
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_RenderFrame(23.25%)</t>
+          <t>Function: cycle_DoSyscall(20.05%)</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
@@ -8097,7 +8097,7 @@
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>Function: cycle_DoSyscall(20.05%)</t>
+          <t>Function: cycle_UpdateScene(16.85%)</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
@@ -8132,124 +8132,124 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F136" s="1" t="inlineStr">
-        <is>
-          <t>Function: cycle_UpdateScene(16.85%)</t>
-        </is>
-      </c>
-      <c r="G136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K136" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L136" s="1" t="inlineStr">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K137" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L137" s="2" t="inlineStr">
+      <c r="A137" s="1" t="inlineStr">
+        <is>
+          <t>UnityMain(43.34%)</t>
+        </is>
+      </c>
+      <c r="B137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C137" s="1" t="inlineStr">
+        <is>
+          <t>Library: libc.so(37%)</t>
+        </is>
+      </c>
+      <c r="D137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F137" s="1" t="inlineStr">
+        <is>
+          <t>Function: fe_UpdateScene(20.25%)</t>
+        </is>
+      </c>
+      <c r="G137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K137" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L137" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -8258,7 +8258,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>UnityMain(43.34%)</t>
+          <t/>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -8268,7 +8268,7 @@
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>Library: libc.so(37%)</t>
+          <t/>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_UpdateScene(20.25%)</t>
+          <t>Function: fe_TextureUpload(17.05%)</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
@@ -8345,7 +8345,7 @@
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_TextureUpload(17.05%)</t>
+          <t>Function: fe_EncodeFrame(13.85%)</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(30%)</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(13.85%)</t>
+          <t>Function: fe_BinderTransact(20.75%)</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(30%)</t>
+          <t/>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
@@ -8469,7 +8469,7 @@
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_BinderTransact(20.75%)</t>
+          <t>Function: fe_PhysicsStep(17.55%)</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_PhysicsStep(17.55%)</t>
+          <t>Function: fe_RenderFrame(14.35%)</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
@@ -8578,7 +8578,7 @@
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(23%)</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_RenderFrame(14.35%)</t>
+          <t>Function: fe_TextureUpload(21.25%)</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
@@ -8640,7 +8640,7 @@
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(23%)</t>
+          <t/>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_TextureUpload(21.25%)</t>
+          <t>Function: fe_EncodeFrame(18.05%)</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(18.05%)</t>
+          <t>Function: fe_ScheduleTask(14.85%)</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
@@ -8754,7 +8754,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>RenderThread(35.39%)</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libGLESv2.so(38.5%)</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(14.85%)</t>
+          <t>Function: fe_TextureUpload(21.25%)</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
@@ -8816,7 +8816,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>RenderThread(35.39%)</t>
+          <t/>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(38.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_TextureUpload(21.25%)</t>
+          <t>Function: fe_EncodeFrame(18.05%)</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(18.05%)</t>
+          <t>Function: fe_ScheduleTask(14.85%)</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(31.5%)</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
@@ -8965,7 +8965,7 @@
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(14.85%)</t>
+          <t>Function: fe_PhysicsStep(21.75%)</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(31.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_PhysicsStep(21.75%)</t>
+          <t>Function: fe_RenderFrame(18.55%)</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
@@ -9089,7 +9089,7 @@
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_RenderFrame(18.55%)</t>
+          <t>Function: fe_DoSyscall(15.35%)</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
@@ -9136,7 +9136,7 @@
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(24.5%)</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
@@ -9151,7 +9151,7 @@
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_DoSyscall(15.35%)</t>
+          <t>Function: fe_EncodeFrame(22.25%)</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
@@ -9198,7 +9198,7 @@
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
@@ -9213,7 +9213,7 @@
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(22.25%)</t>
+          <t>Function: fe_ScheduleTask(19.05%)</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
@@ -9275,7 +9275,7 @@
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(19.05%)</t>
+          <t>Function: fe_WaitFence(15.85%)</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
@@ -9312,7 +9312,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>BinderWorker(27.44%)</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(40%)</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
@@ -9337,7 +9337,7 @@
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_WaitFence(15.85%)</t>
+          <t>Function: fe_EncodeFrame(22.25%)</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
@@ -9374,7 +9374,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>BinderWorker(27.44%)</t>
+          <t/>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(40%)</t>
+          <t/>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_EncodeFrame(22.25%)</t>
+          <t>Function: fe_ScheduleTask(19.05%)</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(19.05%)</t>
+          <t>Function: fe_WaitFence(15.85%)</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
@@ -9508,7 +9508,7 @@
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(33%)</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
@@ -9523,7 +9523,7 @@
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_WaitFence(15.85%)</t>
+          <t>Function: fe_RenderFrame(22.75%)</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(33%)</t>
+          <t/>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_RenderFrame(22.75%)</t>
+          <t>Function: fe_DoSyscall(19.55%)</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_DoSyscall(19.55%)</t>
+          <t>Function: fe_UpdateScene(16.35%)</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
@@ -9694,7 +9694,7 @@
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libhwui.so(26%)</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
@@ -9709,7 +9709,7 @@
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_UpdateScene(16.35%)</t>
+          <t>Function: fe_ScheduleTask(23.25%)</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
@@ -9756,7 +9756,7 @@
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>Library: libhwui.so(26%)</t>
+          <t/>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_ScheduleTask(23.25%)</t>
+          <t>Function: fe_WaitFence(20.05%)</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
@@ -9833,7 +9833,7 @@
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>Function: fe_WaitFence(20.05%)</t>
+          <t>Function: fe_BinderTransact(16.85%)</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
@@ -9868,124 +9868,124 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F164" s="1" t="inlineStr">
-        <is>
-          <t>Function: fe_BinderTransact(16.85%)</t>
-        </is>
-      </c>
-      <c r="G164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K164" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L164" s="1" t="inlineStr">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L164" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="B165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K165" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L165" s="2" t="inlineStr">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t>UnityMain(47.99%)</t>
+        </is>
+      </c>
+      <c r="B165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C165" s="1" t="inlineStr">
+        <is>
+          <t>Library: libGLESv2.so(37%)</t>
+        </is>
+      </c>
+      <c r="D165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F165" s="1" t="inlineStr">
+        <is>
+          <t>Function: be_BinderTransact(20.25%)</t>
+        </is>
+      </c>
+      <c r="G165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K165" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L165" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -9994,7 +9994,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>UnityMain(47.99%)</t>
+          <t/>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>Library: libGLESv2.so(37%)</t>
+          <t/>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
@@ -10019,7 +10019,7 @@
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>Function: be_BinderTransact(20.25%)</t>
+          <t>Function: be_PhysicsStep(17.05%)</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
@@ -10081,7 +10081,7 @@
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>Function: be_PhysicsStep(17.05%)</t>
+          <t>Function: be_RenderFrame(13.85%)</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(30%)</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(13.85%)</t>
+          <t>Function: be_TextureUpload(20.75%)</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(30%)</t>
+          <t/>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
@@ -10205,7 +10205,7 @@
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>Function: be_TextureUpload(20.75%)</t>
+          <t>Function: be_EncodeFrame(17.55%)</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>Function: be_EncodeFrame(17.55%)</t>
+          <t>Function: be_ScheduleTask(14.35%)</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C171" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(23%)</t>
         </is>
       </c>
       <c r="D171" s="1" t="inlineStr">
@@ -10329,7 +10329,7 @@
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>Function: be_ScheduleTask(14.35%)</t>
+          <t>Function: be_PhysicsStep(21.25%)</t>
         </is>
       </c>
       <c r="G171" s="1" t="inlineStr">
@@ -10376,7 +10376,7 @@
       </c>
       <c r="C172" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(23%)</t>
+          <t/>
         </is>
       </c>
       <c r="D172" s="1" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>Function: be_PhysicsStep(21.25%)</t>
+          <t>Function: be_RenderFrame(18.05%)</t>
         </is>
       </c>
       <c r="G172" s="1" t="inlineStr">
@@ -10453,7 +10453,7 @@
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(18.05%)</t>
+          <t>Function: be_DoSyscall(14.85%)</t>
         </is>
       </c>
       <c r="G173" s="1" t="inlineStr">
@@ -10490,7 +10490,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>RenderThread(39.18%)</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="C174" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libbinder.so(38.5%)</t>
         </is>
       </c>
       <c r="D174" s="1" t="inlineStr">
@@ -10515,7 +10515,7 @@
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(14.85%)</t>
+          <t>Function: be_PhysicsStep(21.25%)</t>
         </is>
       </c>
       <c r="G174" s="1" t="inlineStr">
@@ -10552,7 +10552,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>RenderThread(39.18%)</t>
+          <t/>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -10562,7 +10562,7 @@
       </c>
       <c r="C175" s="1" t="inlineStr">
         <is>
-          <t>Library: libbinder.so(38.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D175" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t>Function: be_PhysicsStep(21.25%)</t>
+          <t>Function: be_RenderFrame(18.05%)</t>
         </is>
       </c>
       <c r="G175" s="1" t="inlineStr">
@@ -10639,7 +10639,7 @@
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(18.05%)</t>
+          <t>Function: be_DoSyscall(14.85%)</t>
         </is>
       </c>
       <c r="G176" s="1" t="inlineStr">
@@ -10686,7 +10686,7 @@
       </c>
       <c r="C177" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libcamera_client.so(31.5%)</t>
         </is>
       </c>
       <c r="D177" s="1" t="inlineStr">
@@ -10701,7 +10701,7 @@
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(14.85%)</t>
+          <t>Function: be_EncodeFrame(21.75%)</t>
         </is>
       </c>
       <c r="G177" s="1" t="inlineStr">
@@ -10748,7 +10748,7 @@
       </c>
       <c r="C178" s="1" t="inlineStr">
         <is>
-          <t>Library: libcamera_client.so(31.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D178" s="1" t="inlineStr">
@@ -10763,7 +10763,7 @@
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t>Function: be_EncodeFrame(21.75%)</t>
+          <t>Function: be_ScheduleTask(18.55%)</t>
         </is>
       </c>
       <c r="G178" s="1" t="inlineStr">
@@ -10825,7 +10825,7 @@
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>Function: be_ScheduleTask(18.55%)</t>
+          <t>Function: be_WaitFence(15.35%)</t>
         </is>
       </c>
       <c r="G179" s="1" t="inlineStr">
@@ -10872,7 +10872,7 @@
       </c>
       <c r="C180" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libhwui.so(24.5%)</t>
         </is>
       </c>
       <c r="D180" s="1" t="inlineStr">
@@ -10887,7 +10887,7 @@
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>Function: be_WaitFence(15.35%)</t>
+          <t>Function: be_RenderFrame(22.25%)</t>
         </is>
       </c>
       <c r="G180" s="1" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="C181" s="1" t="inlineStr">
         <is>
-          <t>Library: libhwui.so(24.5%)</t>
+          <t/>
         </is>
       </c>
       <c r="D181" s="1" t="inlineStr">
@@ -10949,7 +10949,7 @@
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(22.25%)</t>
+          <t>Function: be_DoSyscall(19.05%)</t>
         </is>
       </c>
       <c r="G181" s="1" t="inlineStr">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(19.05%)</t>
+          <t>Function: be_UpdateScene(15.85%)</t>
         </is>
       </c>
       <c r="G182" s="1" t="inlineStr">
@@ -11048,7 +11048,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>BinderWorker(30.38%)</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -11058,7 +11058,7 @@
       </c>
       <c r="C183" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libskia.so(40%)</t>
         </is>
       </c>
       <c r="D183" s="1" t="inlineStr">
@@ -11073,7 +11073,7 @@
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>Function: be_UpdateScene(15.85%)</t>
+          <t>Function: be_RenderFrame(22.25%)</t>
         </is>
       </c>
       <c r="G183" s="1" t="inlineStr">
@@ -11110,7 +11110,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>BinderWorker(30.38%)</t>
+          <t/>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="C184" s="1" t="inlineStr">
         <is>
-          <t>Library: libskia.so(40%)</t>
+          <t/>
         </is>
       </c>
       <c r="D184" s="1" t="inlineStr">
@@ -11135,7 +11135,7 @@
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>Function: be_RenderFrame(22.25%)</t>
+          <t>Function: be_DoSyscall(19.05%)</t>
         </is>
       </c>
       <c r="G184" s="1" t="inlineStr">
@@ -11197,7 +11197,7 @@
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(19.05%)</t>
+          <t>Function: be_UpdateScene(15.85%)</t>
         </is>
       </c>
       <c r="G185" s="1" t="inlineStr">
@@ -11244,7 +11244,7 @@
       </c>
       <c r="C186" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libunity.so(33%)</t>
         </is>
       </c>
       <c r="D186" s="1" t="inlineStr">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>Function: be_UpdateScene(15.85%)</t>
+          <t>Function: be_ScheduleTask(22.75%)</t>
         </is>
       </c>
       <c r="G186" s="1" t="inlineStr">
@@ -11306,7 +11306,7 @@
       </c>
       <c r="C187" s="1" t="inlineStr">
         <is>
-          <t>Library: libunity.so(33%)</t>
+          <t/>
         </is>
       </c>
       <c r="D187" s="1" t="inlineStr">
@@ -11321,7 +11321,7 @@
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>Function: be_ScheduleTask(22.75%)</t>
+          <t>Function: be_WaitFence(19.55%)</t>
         </is>
       </c>
       <c r="G187" s="1" t="inlineStr">
@@ -11383,7 +11383,7 @@
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>Function: be_WaitFence(19.55%)</t>
+          <t>Function: be_BinderTransact(16.35%)</t>
         </is>
       </c>
       <c r="G188" s="1" t="inlineStr">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="C189" s="1" t="inlineStr">
         <is>
-          <t/>
+          <t>Library: libart.so(26%)</t>
         </is>
       </c>
       <c r="D189" s="1" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>Function: be_BinderTransact(16.35%)</t>
+          <t>Function: be_DoSyscall(23.25%)</t>
         </is>
       </c>
       <c r="G189" s="1" t="inlineStr">
@@ -11492,7 +11492,7 @@
       </c>
       <c r="C190" s="1" t="inlineStr">
         <is>
-          <t>Library: libart.so(26%)</t>
+          <t/>
         </is>
       </c>
       <c r="D190" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>Function: be_DoSyscall(23.25%)</t>
+          <t>Function: be_UpdateScene(20.05%)</t>
         </is>
       </c>
       <c r="G190" s="1" t="inlineStr">
@@ -11569,7 +11569,7 @@
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>Function: be_UpdateScene(20.05%)</t>
+          <t>Function: be_TextureUpload(16.85%)</t>
         </is>
       </c>
       <c r="G191" s="1" t="inlineStr">
@@ -11603,70 +11603,8 @@
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F192" s="1" t="inlineStr">
-        <is>
-          <t>Function: be_TextureUpload(16.85%)</t>
-        </is>
-      </c>
-      <c r="G192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L192" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="94">
+  <mergeCells count="92">
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:D3"/>
@@ -11710,57 +11648,55 @@
     <mergeCell ref="A79:L79"/>
     <mergeCell ref="A80:D80"/>
     <mergeCell ref="E80:H80"/>
-    <mergeCell ref="A88:L88"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="E89:H89"/>
-    <mergeCell ref="A96:L96"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="E97:H97"/>
+    <mergeCell ref="A87:L87"/>
+    <mergeCell ref="A88:D88"/>
+    <mergeCell ref="E88:H88"/>
+    <mergeCell ref="A95:L95"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="E96:H96"/>
     <mergeCell ref="A103:L103"/>
     <mergeCell ref="A104:B104"/>
     <mergeCell ref="A105:B105"/>
     <mergeCell ref="A106:B106"/>
-    <mergeCell ref="A107:B107"/>
     <mergeCell ref="A108:L108"/>
-    <mergeCell ref="A109:L109"/>
-    <mergeCell ref="C110:E112"/>
-    <mergeCell ref="C113:E115"/>
-    <mergeCell ref="C116:E118"/>
-    <mergeCell ref="A110:B118"/>
-    <mergeCell ref="C119:E121"/>
-    <mergeCell ref="C122:E124"/>
-    <mergeCell ref="C125:E127"/>
-    <mergeCell ref="A119:B127"/>
-    <mergeCell ref="C128:E130"/>
-    <mergeCell ref="C131:E133"/>
-    <mergeCell ref="C134:E136"/>
-    <mergeCell ref="A128:B136"/>
-    <mergeCell ref="A137:L137"/>
-    <mergeCell ref="C138:E140"/>
-    <mergeCell ref="C141:E143"/>
-    <mergeCell ref="C144:E146"/>
-    <mergeCell ref="A138:B146"/>
-    <mergeCell ref="C147:E149"/>
-    <mergeCell ref="C150:E152"/>
-    <mergeCell ref="C153:E155"/>
-    <mergeCell ref="A147:B155"/>
-    <mergeCell ref="C156:E158"/>
-    <mergeCell ref="C159:E161"/>
-    <mergeCell ref="C162:E164"/>
-    <mergeCell ref="A156:B164"/>
-    <mergeCell ref="A165:L165"/>
-    <mergeCell ref="C166:E168"/>
-    <mergeCell ref="C169:E171"/>
-    <mergeCell ref="C172:E174"/>
-    <mergeCell ref="A166:B174"/>
-    <mergeCell ref="C175:E177"/>
-    <mergeCell ref="C178:E180"/>
-    <mergeCell ref="C181:E183"/>
-    <mergeCell ref="A175:B183"/>
-    <mergeCell ref="C184:E186"/>
-    <mergeCell ref="C187:E189"/>
-    <mergeCell ref="C190:E192"/>
-    <mergeCell ref="A184:B192"/>
+    <mergeCell ref="C109:E111"/>
+    <mergeCell ref="C112:E114"/>
+    <mergeCell ref="C115:E117"/>
+    <mergeCell ref="A109:B117"/>
+    <mergeCell ref="C118:E120"/>
+    <mergeCell ref="C121:E123"/>
+    <mergeCell ref="C124:E126"/>
+    <mergeCell ref="A118:B126"/>
+    <mergeCell ref="C127:E129"/>
+    <mergeCell ref="C130:E132"/>
+    <mergeCell ref="C133:E135"/>
+    <mergeCell ref="A127:B135"/>
+    <mergeCell ref="A136:L136"/>
+    <mergeCell ref="C137:E139"/>
+    <mergeCell ref="C140:E142"/>
+    <mergeCell ref="C143:E145"/>
+    <mergeCell ref="A137:B145"/>
+    <mergeCell ref="C146:E148"/>
+    <mergeCell ref="C149:E151"/>
+    <mergeCell ref="C152:E154"/>
+    <mergeCell ref="A146:B154"/>
+    <mergeCell ref="C155:E157"/>
+    <mergeCell ref="C158:E160"/>
+    <mergeCell ref="C161:E163"/>
+    <mergeCell ref="A155:B163"/>
+    <mergeCell ref="A164:L164"/>
+    <mergeCell ref="C165:E167"/>
+    <mergeCell ref="C168:E170"/>
+    <mergeCell ref="C171:E173"/>
+    <mergeCell ref="A165:B173"/>
+    <mergeCell ref="C174:E176"/>
+    <mergeCell ref="C177:E179"/>
+    <mergeCell ref="C180:E182"/>
+    <mergeCell ref="A174:B182"/>
+    <mergeCell ref="C183:E185"/>
+    <mergeCell ref="C186:E188"/>
+    <mergeCell ref="C189:E191"/>
+    <mergeCell ref="A183:B191"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Align instruction and hotspot import coordinates
</commit_message>
<xml_diff>
--- a/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
+++ b/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
@@ -4724,107 +4724,99 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>UnityMain线程</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I79" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J79" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K79" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L79" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>Kernel</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G80" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H80" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="B80" s="5">
+        <v>2.12</v>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D80" s="5">
+        <v>3.98</v>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="F80" s="5">
+        <v>0.72</v>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="H80" s="5">
+        <v>1.38</v>
       </c>
       <c r="I80" s="1" t="inlineStr">
         <is>
@@ -4850,11 +4842,11 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="B81" s="5">
-        <v>2.12</v>
+        <v>2.43</v>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
@@ -4866,11 +4858,11 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="F81" s="5">
-        <v>0.72</v>
+        <v>0.83</v>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
@@ -4904,35 +4896,35 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B82" s="5">
-        <v>2.43</v>
+        <v>2.74</v>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="D82" s="5">
-        <v>3.98</v>
+        <v>4.91</v>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F82" s="5">
-        <v>0.83</v>
+        <v>0.94</v>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="H82" s="5">
-        <v>1.38</v>
+        <v>1.71</v>
       </c>
       <c r="I82" s="1" t="inlineStr">
         <is>
@@ -4958,35 +4950,35 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B83" s="5">
-        <v>2.74</v>
+        <v>3.05</v>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="D83" s="5">
-        <v>4.91</v>
+        <v>4.6</v>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F83" s="5">
-        <v>0.94</v>
+        <v>1.05</v>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="H83" s="5">
-        <v>1.71</v>
+        <v>1.6</v>
       </c>
       <c r="I83" s="1" t="inlineStr">
         <is>
@@ -5020,11 +5012,13 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D84" s="5">
-        <v>4.6</v>
+          <t/>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
@@ -5036,11 +5030,13 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H84" s="5">
-        <v>1.6</v>
+          <t/>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I84" s="1" t="inlineStr">
         <is>
@@ -5074,11 +5070,13 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D85" s="5">
-        <v>3.05</v>
+          <t/>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
@@ -5090,11 +5088,13 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H85" s="5">
-        <v>1.05</v>
+          <t/>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I85" s="1" t="inlineStr">
         <is>
@@ -5180,107 +5180,99 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
+      <c r="A87" s="3" t="inlineStr">
         <is>
           <t>RenderThread线程</t>
         </is>
       </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K87" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L87" s="2" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I87" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J87" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K87" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L87" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C88" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>Kernel</t>
-        </is>
-      </c>
-      <c r="F88" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G88" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H88" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="B88" s="5">
+        <v>2.6</v>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D88" s="5">
+        <v>4.46</v>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="F88" s="5">
+        <v>0.89</v>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="H88" s="5">
+        <v>1.55</v>
       </c>
       <c r="I88" s="1" t="inlineStr">
         <is>
@@ -5306,11 +5298,11 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="B89" s="5">
-        <v>2.6</v>
+        <v>2.91</v>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
@@ -5322,11 +5314,11 @@
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="F89" s="5">
-        <v>0.89</v>
+        <v>1</v>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
@@ -5360,35 +5352,35 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B90" s="5">
-        <v>2.91</v>
+        <v>3.22</v>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="D90" s="5">
-        <v>4.46</v>
+        <v>5.39</v>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F90" s="5">
-        <v>1</v>
+        <v>1.11</v>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="H90" s="5">
-        <v>1.55</v>
+        <v>1.88</v>
       </c>
       <c r="I90" s="1" t="inlineStr">
         <is>
@@ -5414,35 +5406,35 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B91" s="5">
-        <v>3.22</v>
+        <v>3.53</v>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="D91" s="5">
-        <v>5.39</v>
+        <v>5.08</v>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F91" s="5">
-        <v>1.11</v>
+        <v>1.22</v>
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="H91" s="5">
-        <v>1.88</v>
+        <v>1.77</v>
       </c>
       <c r="I91" s="1" t="inlineStr">
         <is>
@@ -5476,11 +5468,13 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D92" s="5">
-        <v>5.08</v>
+          <t/>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
@@ -5492,11 +5486,13 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H92" s="5">
-        <v>1.77</v>
+          <t/>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I92" s="1" t="inlineStr">
         <is>
@@ -5530,11 +5526,13 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D93" s="5">
-        <v>3.53</v>
+          <t/>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
@@ -5546,11 +5544,13 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H93" s="5">
-        <v>1.22</v>
+          <t/>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I93" s="1" t="inlineStr">
         <is>
@@ -5636,107 +5636,99 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="inlineStr">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>BinderWorker线程</t>
         </is>
       </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K95" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L95" s="2" t="inlineStr">
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I95" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J95" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K95" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L95" s="1" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
-        <is>
-          <t>Kernel</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G96" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H96" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="B96" s="5">
+        <v>3.08</v>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="D96" s="5">
+        <v>4.94</v>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>LD/ST_RETIRED_PKI</t>
+        </is>
+      </c>
+      <c r="F96" s="5">
+        <v>1.06</v>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>LD/STREX_SPEC_PKI</t>
+        </is>
+      </c>
+      <c r="H96" s="5">
+        <v>1.72</v>
       </c>
       <c r="I96" s="1" t="inlineStr">
         <is>
@@ -5762,11 +5754,11 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="B97" s="5">
-        <v>3.08</v>
+        <v>3.39</v>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
@@ -5778,11 +5770,11 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>LD/ST_RETIRED_PKI</t>
+          <t>BR_RETIRED_PKI</t>
         </is>
       </c>
       <c r="F97" s="5">
-        <v>1.06</v>
+        <v>1.17</v>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
@@ -5816,35 +5808,35 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B98" s="5">
-        <v>3.39</v>
+        <v>3.7</v>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="D98" s="5">
-        <v>4.94</v>
+        <v>5.87</v>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>BR_RETIRED_PKI</t>
+          <t>DP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F98" s="5">
-        <v>1.17</v>
+        <v>1.28</v>
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>LD/STREX_SPEC_PKI</t>
+          <t>UNALIGNED_LDST_SPEC_PKI</t>
         </is>
       </c>
       <c r="H98" s="5">
-        <v>1.72</v>
+        <v>2.05</v>
       </c>
       <c r="I98" s="1" t="inlineStr">
         <is>
@@ -5870,35 +5862,35 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="B99" s="5">
-        <v>3.7</v>
+        <v>4.01</v>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="D99" s="5">
-        <v>5.87</v>
+        <v>5.56</v>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>DP_SPEC_PKI</t>
+          <t>VFP_SPEC_PKI</t>
         </is>
       </c>
       <c r="F99" s="5">
-        <v>1.28</v>
+        <v>1.39</v>
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>UNALIGNED_LDST_SPEC_PKI</t>
+          <t>BARRIER_SPEC_PKI</t>
         </is>
       </c>
       <c r="H99" s="5">
-        <v>2.05</v>
+        <v>1.94</v>
       </c>
       <c r="I99" s="1" t="inlineStr">
         <is>
@@ -5932,11 +5924,13 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D100" s="5">
-        <v>5.56</v>
+          <t/>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
@@ -5948,11 +5942,13 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>BARRIER_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H100" s="5">
-        <v>1.94</v>
+          <t/>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I100" s="1" t="inlineStr">
         <is>
@@ -5986,11 +5982,13 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="D101" s="5">
-        <v>4.01</v>
+          <t/>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
@@ -6002,11 +6000,13 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>VFP_SPEC_PKI</t>
-        </is>
-      </c>
-      <c r="H101" s="5">
-        <v>1.39</v>
+          <t/>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="I101" s="1" t="inlineStr">
         <is>
@@ -11604,7 +11604,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="92">
+  <mergeCells count="83">
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:D3"/>
@@ -11645,15 +11645,6 @@
     <mergeCell ref="A64:L64"/>
     <mergeCell ref="A74:L74"/>
     <mergeCell ref="A78:L78"/>
-    <mergeCell ref="A79:L79"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="E80:H80"/>
-    <mergeCell ref="A87:L87"/>
-    <mergeCell ref="A88:D88"/>
-    <mergeCell ref="E88:H88"/>
-    <mergeCell ref="A95:L95"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="E96:H96"/>
     <mergeCell ref="A103:L103"/>
     <mergeCell ref="A104:B104"/>
     <mergeCell ref="A105:B105"/>

</xml_diff>

<commit_message>
Improve metric import precision and hotspot diagnostics
</commit_message>
<xml_diff>
--- a/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
+++ b/source_data/01_game/qqfeiche_replay/CPU测试场景库分析_qqfeiche_replay.xlsx
@@ -4664,7 +4664,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>4. 指令分布</t>
+          <t>UnityMain线程</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4726,12 +4726,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>UnityMain线程</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t/>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -5118,62 +5118,62 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K86" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L86" s="1" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>RenderThread线程</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -5182,12 +5182,12 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>RenderThread线程</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t/>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -5574,62 +5574,62 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K94" s="1" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L94" s="1" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>BinderWorker线程</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -5638,12 +5638,12 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>BinderWorker线程</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t/>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="83">
+  <mergeCells count="92">
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:D3"/>
@@ -11645,6 +11645,15 @@
     <mergeCell ref="A64:L64"/>
     <mergeCell ref="A74:L74"/>
     <mergeCell ref="A78:L78"/>
+    <mergeCell ref="A78:L78"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="E79:H79"/>
+    <mergeCell ref="A86:L86"/>
+    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="E87:H87"/>
+    <mergeCell ref="A94:L94"/>
+    <mergeCell ref="A95:D95"/>
+    <mergeCell ref="E95:H95"/>
     <mergeCell ref="A103:L103"/>
     <mergeCell ref="A104:B104"/>
     <mergeCell ref="A105:B105"/>

</xml_diff>